<commit_message>
Updated time estimates for 6.0 / 7,0
</commit_message>
<xml_diff>
--- a/Documentation/Materiale til brug ved fondsansøgninger/Version 6.0/Tidsestimater.2023.12.05.xlsx
+++ b/Documentation/Materiale til brug ved fondsansøgninger/Version 6.0/Tidsestimater.2023.12.05.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Oversigt" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="74">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -33,13 +33,16 @@
     <t xml:space="preserve">Del-System</t>
   </si>
   <si>
-    <t xml:space="preserve">Dage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ansøgning 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ansøgning 2</t>
+    <t xml:space="preserve">Arbejdsdage
+Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arbejdsdage
+Ansøgning 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arbejdsdage
+Ansøgning 2</t>
   </si>
   <si>
     <t xml:space="preserve">Udsat</t>
@@ -243,7 +246,7 @@
     <t xml:space="preserve">Total antal arbejdsdage @7,5 timer</t>
   </si>
   <si>
-    <t xml:space="preserve">Total antal arbejdstimer</t>
+    <t xml:space="preserve">Arbejdsdage</t>
   </si>
 </sst>
 </file>
@@ -326,7 +329,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -339,7 +342,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -365,12 +372,12 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="75.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -380,13 +387,13 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -412,7 +419,7 @@
       <c r="F2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="3"/>
+      <c r="G2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
@@ -433,7 +440,7 @@
       <c r="F3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -454,7 +461,7 @@
       <c r="F4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="3"/>
+      <c r="G4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -475,7 +482,7 @@
       <c r="F5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="3"/>
+      <c r="G5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -519,7 +526,7 @@
       <c r="F7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="3"/>
+      <c r="G7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
@@ -540,7 +547,7 @@
       <c r="F8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="3"/>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
@@ -561,7 +568,7 @@
       <c r="F9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="3"/>
+      <c r="G9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
@@ -582,7 +589,7 @@
       <c r="F10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="3"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
@@ -603,7 +610,7 @@
       <c r="F11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="3"/>
+      <c r="G11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
@@ -624,7 +631,7 @@
       <c r="F12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="3"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
@@ -691,7 +698,7 @@
       <c r="F15" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="3"/>
+      <c r="G15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
@@ -735,7 +742,7 @@
       <c r="F17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G17" s="3"/>
+      <c r="G17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
@@ -779,7 +786,7 @@
       <c r="F19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="3"/>
+      <c r="G19" s="4"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
@@ -800,7 +807,7 @@
       <c r="F20" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G20" s="3"/>
+      <c r="G20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
@@ -913,7 +920,7 @@
       <c r="F25" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="3"/>
+      <c r="G25" s="4"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
@@ -930,7 +937,7 @@
       <c r="F26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="3"/>
+      <c r="G26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
@@ -951,7 +958,7 @@
       <c r="F27" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G27" s="3"/>
+      <c r="G27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
@@ -1014,7 +1021,7 @@
       <c r="F30" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="G30" s="4" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1035,10 +1042,10 @@
       <c r="F31" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="3"/>
+      <c r="G31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3"/>
+      <c r="A32" s="4"/>
       <c r="B32" s="2" t="s">
         <v>72</v>
       </c>
@@ -1052,25 +1059,9 @@
         <f aca="false">SUM(F2:F31)</f>
         <v>18</v>
       </c>
-      <c r="G32" s="3"/>
-    </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3"/>
-      <c r="B33" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2" t="n">
-        <f aca="false">E32*7.5</f>
-        <v>135</v>
-      </c>
-      <c r="F33" s="2" t="n">
-        <f aca="false">F32*7.5</f>
-        <v>135</v>
-      </c>
-      <c r="G33" s="3"/>
-    </row>
+      <c r="G32" s="4"/>
+    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1088,13 +1079,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D1048576"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="75.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.79"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1108,7 +1099,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1266,7 +1257,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3"/>
+      <c r="A13" s="4"/>
       <c r="B13" s="2" t="s">
         <v>72</v>
       </c>
@@ -1276,17 +1267,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="B14" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2" t="n">
-        <f aca="false">D13*7.5</f>
-        <v>135</v>
-      </c>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1306,7 +1287,7 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="75.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.1"/>
@@ -1323,7 +1304,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1411,7 +1392,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
+      <c r="A8" s="4"/>
       <c r="B8" s="2" t="s">
         <v>72</v>
       </c>
@@ -1422,15 +1403,10 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3"/>
-      <c r="B9" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="A9" s="4"/>
+      <c r="B9" s="2"/>
       <c r="C9" s="2"/>
-      <c r="D9" s="2" t="n">
-        <f aca="false">D8*7.5</f>
-        <v>135</v>
-      </c>
+      <c r="D9" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>